<commit_message>
Refactor evaluation metrics into Two-Tier Framework: drop Scheme 1, unify boundary and misclassification into Category C (0.5 credit), restrict S to non-overlapping FPs
</commit_message>
<xml_diff>
--- a/publication/results/bert_runs_FAERS_LOO/loo_evaluation_summary.xlsx
+++ b/publication/results/bert_runs_FAERS_LOO/loo_evaluation_summary.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="All_Runs_Per_Seed" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Fold_Summary_Across_Seeds" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Per_Category_Summary" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Bootstrap_95CI" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All_Runs_Per_Seed" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fold_Summary_Across_Seeds" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Per_Category_Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,13 +19,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +39,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -45,12 +47,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -420,84 +431,84 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>fold</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>fold_name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>seed</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>test_case_series</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>S_wrong_class</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>C_boundary</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>C_class</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>C_total</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>S_non_overlap</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>strict_P</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>strict_R</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>strict_F1</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>ade_P</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>ade_R</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>ade_F1</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>detection_F1</t>
         </is>
       </c>
     </row>
@@ -528,31 +539,31 @@
         <v>890</v>
       </c>
       <c r="H2" t="n">
+        <v>1962</v>
+      </c>
+      <c r="I2" t="n">
         <v>3084</v>
       </c>
-      <c r="I2" t="n">
+      <c r="J2" t="n">
         <v>1198</v>
       </c>
-      <c r="J2" t="n">
+      <c r="K2" t="n">
         <v>0.5545</v>
       </c>
-      <c r="K2" t="n">
-        <v>0.7345</v>
-      </c>
       <c r="L2" t="n">
-        <v>0.6319</v>
+        <v>0.6653</v>
       </c>
       <c r="M2" t="n">
-        <v>0.8167</v>
+        <v>0.6048</v>
       </c>
       <c r="N2" t="n">
-        <v>0.7972</v>
+        <v>0.8056</v>
       </c>
       <c r="O2" t="n">
-        <v>0.8068</v>
+        <v>0.7692</v>
       </c>
       <c r="P2" t="n">
-        <v>0.8933</v>
+        <v>0.787</v>
       </c>
     </row>
     <row r="3">
@@ -582,31 +593,31 @@
         <v>849</v>
       </c>
       <c r="H3" t="n">
+        <v>1723</v>
+      </c>
+      <c r="I3" t="n">
         <v>2648</v>
       </c>
-      <c r="I3" t="n">
+      <c r="J3" t="n">
         <v>1677</v>
       </c>
-      <c r="J3" t="n">
+      <c r="K3" t="n">
         <v>0.5802</v>
       </c>
-      <c r="K3" t="n">
-        <v>0.7030999999999999</v>
-      </c>
       <c r="L3" t="n">
-        <v>0.6357</v>
+        <v>0.6398</v>
       </c>
       <c r="M3" t="n">
-        <v>0.8316</v>
+        <v>0.6085</v>
       </c>
       <c r="N3" t="n">
-        <v>0.7539</v>
+        <v>0.8192</v>
       </c>
       <c r="O3" t="n">
-        <v>0.7909</v>
+        <v>0.7311</v>
       </c>
       <c r="P3" t="n">
-        <v>0.8691</v>
+        <v>0.7726</v>
       </c>
     </row>
     <row r="4">
@@ -636,31 +647,31 @@
         <v>810</v>
       </c>
       <c r="H4" t="n">
+        <v>1697</v>
+      </c>
+      <c r="I4" t="n">
         <v>2615</v>
       </c>
-      <c r="I4" t="n">
+      <c r="J4" t="n">
         <v>1686</v>
       </c>
-      <c r="J4" t="n">
+      <c r="K4" t="n">
         <v>0.5841</v>
       </c>
-      <c r="K4" t="n">
-        <v>0.7019</v>
-      </c>
       <c r="L4" t="n">
-        <v>0.6375999999999999</v>
+        <v>0.6415999999999999</v>
       </c>
       <c r="M4" t="n">
-        <v>0.8334</v>
+        <v>0.6115</v>
       </c>
       <c r="N4" t="n">
-        <v>0.7532</v>
+        <v>0.8213</v>
       </c>
       <c r="O4" t="n">
-        <v>0.7913</v>
+        <v>0.7315</v>
       </c>
       <c r="P4" t="n">
-        <v>0.8689</v>
+        <v>0.7738</v>
       </c>
     </row>
     <row r="5">
@@ -690,31 +701,31 @@
         <v>1725</v>
       </c>
       <c r="H5" t="n">
+        <v>3930</v>
+      </c>
+      <c r="I5" t="n">
         <v>4126</v>
       </c>
-      <c r="I5" t="n">
+      <c r="J5" t="n">
         <v>2309</v>
       </c>
-      <c r="J5" t="n">
+      <c r="K5" t="n">
         <v>0.4839</v>
       </c>
-      <c r="K5" t="n">
-        <v>0.6259</v>
-      </c>
       <c r="L5" t="n">
-        <v>0.5458</v>
+        <v>0.5476</v>
       </c>
       <c r="M5" t="n">
-        <v>0.7714</v>
+        <v>0.5138</v>
       </c>
       <c r="N5" t="n">
-        <v>0.7173</v>
+        <v>0.7605</v>
       </c>
       <c r="O5" t="n">
-        <v>0.7433</v>
+        <v>0.6901</v>
       </c>
       <c r="P5" t="n">
-        <v>0.873</v>
+        <v>0.7236</v>
       </c>
     </row>
     <row r="6">
@@ -744,31 +755,31 @@
         <v>981</v>
       </c>
       <c r="H6" t="n">
+        <v>1908</v>
+      </c>
+      <c r="I6" t="n">
         <v>2777</v>
       </c>
-      <c r="I6" t="n">
+      <c r="J6" t="n">
         <v>1676</v>
       </c>
-      <c r="J6" t="n">
+      <c r="K6" t="n">
         <v>0.5555</v>
       </c>
-      <c r="K6" t="n">
-        <v>0.6923</v>
-      </c>
       <c r="L6" t="n">
-        <v>0.6163999999999999</v>
+        <v>0.6203</v>
       </c>
       <c r="M6" t="n">
-        <v>0.8183</v>
+        <v>0.5862000000000001</v>
       </c>
       <c r="N6" t="n">
-        <v>0.7471</v>
+        <v>0.8051</v>
       </c>
       <c r="O6" t="n">
-        <v>0.7811</v>
+        <v>0.7214</v>
       </c>
       <c r="P6" t="n">
-        <v>0.8676</v>
+        <v>0.761</v>
       </c>
     </row>
     <row r="7">
@@ -798,31 +809,31 @@
         <v>145</v>
       </c>
       <c r="H7" t="n">
+        <v>431</v>
+      </c>
+      <c r="I7" t="n">
         <v>529</v>
       </c>
-      <c r="I7" t="n">
+      <c r="J7" t="n">
         <v>542</v>
       </c>
-      <c r="J7" t="n">
+      <c r="K7" t="n">
         <v>0.6206</v>
       </c>
-      <c r="K7" t="n">
-        <v>0.6546999999999999</v>
-      </c>
       <c r="L7" t="n">
-        <v>0.6372</v>
+        <v>0.6173999999999999</v>
       </c>
       <c r="M7" t="n">
-        <v>0.8461</v>
+        <v>0.619</v>
       </c>
       <c r="N7" t="n">
-        <v>0.7143</v>
+        <v>0.837</v>
       </c>
       <c r="O7" t="n">
-        <v>0.7747000000000001</v>
+        <v>0.7020999999999999</v>
       </c>
       <c r="P7" t="n">
-        <v>0.8558</v>
+        <v>0.7635999999999999</v>
       </c>
     </row>
     <row r="8">
@@ -852,31 +863,31 @@
         <v>1547</v>
       </c>
       <c r="H8" t="n">
+        <v>3669</v>
+      </c>
+      <c r="I8" t="n">
         <v>3731</v>
       </c>
-      <c r="I8" t="n">
+      <c r="J8" t="n">
         <v>2548</v>
       </c>
-      <c r="J8" t="n">
+      <c r="K8" t="n">
         <v>0.5058</v>
       </c>
-      <c r="K8" t="n">
-        <v>0.6186</v>
-      </c>
       <c r="L8" t="n">
-        <v>0.5565</v>
+        <v>0.5492</v>
       </c>
       <c r="M8" t="n">
-        <v>0.7839</v>
+        <v>0.5266</v>
       </c>
       <c r="N8" t="n">
-        <v>0.7052</v>
+        <v>0.7727000000000001</v>
       </c>
       <c r="O8" t="n">
-        <v>0.7425</v>
+        <v>0.6822</v>
       </c>
       <c r="P8" t="n">
-        <v>0.866</v>
+        <v>0.7247</v>
       </c>
     </row>
     <row r="9">
@@ -906,31 +917,31 @@
         <v>154</v>
       </c>
       <c r="H9" t="n">
+        <v>414</v>
+      </c>
+      <c r="I9" t="n">
         <v>523</v>
       </c>
-      <c r="I9" t="n">
+      <c r="J9" t="n">
         <v>539</v>
       </c>
-      <c r="J9" t="n">
+      <c r="K9" t="n">
         <v>0.6292</v>
       </c>
-      <c r="K9" t="n">
-        <v>0.6656</v>
-      </c>
       <c r="L9" t="n">
-        <v>0.6469</v>
+        <v>0.6252</v>
       </c>
       <c r="M9" t="n">
-        <v>0.8518</v>
+        <v>0.6272</v>
       </c>
       <c r="N9" t="n">
-        <v>0.72</v>
+        <v>0.8418</v>
       </c>
       <c r="O9" t="n">
-        <v>0.7804</v>
+        <v>0.7066</v>
       </c>
       <c r="P9" t="n">
-        <v>0.8568</v>
+        <v>0.7683</v>
       </c>
     </row>
     <row r="10">
@@ -960,31 +971,31 @@
         <v>1692</v>
       </c>
       <c r="H10" t="n">
+        <v>3562</v>
+      </c>
+      <c r="I10" t="n">
         <v>3569</v>
       </c>
-      <c r="I10" t="n">
+      <c r="J10" t="n">
         <v>2549</v>
       </c>
-      <c r="J10" t="n">
+      <c r="K10" t="n">
         <v>0.5185</v>
       </c>
-      <c r="K10" t="n">
-        <v>0.6348</v>
-      </c>
       <c r="L10" t="n">
-        <v>0.5708</v>
+        <v>0.5569</v>
       </c>
       <c r="M10" t="n">
-        <v>0.7929</v>
+        <v>0.537</v>
       </c>
       <c r="N10" t="n">
-        <v>0.712</v>
+        <v>0.7796999999999999</v>
       </c>
       <c r="O10" t="n">
-        <v>0.7503</v>
+        <v>0.6860000000000001</v>
       </c>
       <c r="P10" t="n">
-        <v>0.8673</v>
+        <v>0.7299</v>
       </c>
     </row>
     <row r="11">
@@ -1014,31 +1025,31 @@
         <v>951</v>
       </c>
       <c r="H11" t="n">
+        <v>1904</v>
+      </c>
+      <c r="I11" t="n">
         <v>3195</v>
       </c>
-      <c r="I11" t="n">
+      <c r="J11" t="n">
         <v>1451</v>
       </c>
-      <c r="J11" t="n">
+      <c r="K11" t="n">
         <v>0.5441</v>
       </c>
-      <c r="K11" t="n">
-        <v>0.7168</v>
-      </c>
       <c r="L11" t="n">
-        <v>0.6186</v>
+        <v>0.6446</v>
       </c>
       <c r="M11" t="n">
-        <v>0.8126</v>
+        <v>0.5901</v>
       </c>
       <c r="N11" t="n">
-        <v>0.7729</v>
+        <v>0.8008</v>
       </c>
       <c r="O11" t="n">
-        <v>0.7923</v>
+        <v>0.7454</v>
       </c>
       <c r="P11" t="n">
-        <v>0.8766</v>
+        <v>0.7721</v>
       </c>
     </row>
     <row r="12">
@@ -1068,31 +1079,31 @@
         <v>1406</v>
       </c>
       <c r="H12" t="n">
+        <v>3437</v>
+      </c>
+      <c r="I12" t="n">
         <v>3251</v>
       </c>
-      <c r="I12" t="n">
+      <c r="J12" t="n">
         <v>2889</v>
       </c>
-      <c r="J12" t="n">
+      <c r="K12" t="n">
         <v>0.5275</v>
       </c>
-      <c r="K12" t="n">
-        <v>0.6027</v>
-      </c>
       <c r="L12" t="n">
-        <v>0.5626</v>
+        <v>0.5413</v>
       </c>
       <c r="M12" t="n">
-        <v>0.7955</v>
+        <v>0.5343</v>
       </c>
       <c r="N12" t="n">
-        <v>0.6847</v>
+        <v>0.7839</v>
       </c>
       <c r="O12" t="n">
-        <v>0.736</v>
+        <v>0.6659</v>
       </c>
       <c r="P12" t="n">
-        <v>0.8549</v>
+        <v>0.7201</v>
       </c>
     </row>
     <row r="13">
@@ -1122,31 +1133,31 @@
         <v>148</v>
       </c>
       <c r="H13" t="n">
+        <v>363</v>
+      </c>
+      <c r="I13" t="n">
         <v>483</v>
       </c>
-      <c r="I13" t="n">
+      <c r="J13" t="n">
         <v>498</v>
       </c>
-      <c r="J13" t="n">
+      <c r="K13" t="n">
         <v>0.6653</v>
       </c>
-      <c r="K13" t="n">
-        <v>0.7023</v>
-      </c>
       <c r="L13" t="n">
-        <v>0.6833</v>
+        <v>0.6614</v>
       </c>
       <c r="M13" t="n">
-        <v>0.8709</v>
+        <v>0.6634</v>
       </c>
       <c r="N13" t="n">
-        <v>0.7472</v>
+        <v>0.8604000000000001</v>
       </c>
       <c r="O13" t="n">
-        <v>0.8043</v>
+        <v>0.7328</v>
       </c>
       <c r="P13" t="n">
-        <v>0.8686</v>
+        <v>0.7915</v>
       </c>
     </row>
     <row r="14">
@@ -1176,31 +1187,31 @@
         <v>302</v>
       </c>
       <c r="H14" t="n">
+        <v>928</v>
+      </c>
+      <c r="I14" t="n">
         <v>1728</v>
       </c>
-      <c r="I14" t="n">
+      <c r="J14" t="n">
         <v>1165</v>
       </c>
-      <c r="J14" t="n">
+      <c r="K14" t="n">
         <v>0.4926</v>
       </c>
-      <c r="K14" t="n">
-        <v>0.5901999999999999</v>
-      </c>
       <c r="L14" t="n">
-        <v>0.537</v>
+        <v>0.552</v>
       </c>
       <c r="M14" t="n">
-        <v>0.779</v>
+        <v>0.5206</v>
       </c>
       <c r="N14" t="n">
-        <v>0.6618000000000001</v>
+        <v>0.7725</v>
       </c>
       <c r="O14" t="n">
-        <v>0.7156</v>
+        <v>0.6513</v>
       </c>
       <c r="P14" t="n">
-        <v>0.8145</v>
+        <v>0.7068</v>
       </c>
     </row>
     <row r="15">
@@ -1230,31 +1241,31 @@
         <v>143</v>
       </c>
       <c r="H15" t="n">
+        <v>400</v>
+      </c>
+      <c r="I15" t="n">
         <v>468</v>
       </c>
-      <c r="I15" t="n">
+      <c r="J15" t="n">
         <v>491</v>
       </c>
-      <c r="J15" t="n">
+      <c r="K15" t="n">
         <v>0.6556</v>
       </c>
-      <c r="K15" t="n">
-        <v>0.6883</v>
-      </c>
       <c r="L15" t="n">
-        <v>0.6715</v>
+        <v>0.6496</v>
       </c>
       <c r="M15" t="n">
-        <v>0.8636</v>
+        <v>0.6526</v>
       </c>
       <c r="N15" t="n">
-        <v>0.7419</v>
+        <v>0.8538</v>
       </c>
       <c r="O15" t="n">
-        <v>0.7981</v>
+        <v>0.7282999999999999</v>
       </c>
       <c r="P15" t="n">
-        <v>0.871</v>
+        <v>0.7861</v>
       </c>
     </row>
     <row r="16">
@@ -1284,31 +1295,31 @@
         <v>380</v>
       </c>
       <c r="H16" t="n">
+        <v>1091</v>
+      </c>
+      <c r="I16" t="n">
         <v>2342</v>
       </c>
-      <c r="I16" t="n">
+      <c r="J16" t="n">
         <v>821</v>
       </c>
-      <c r="J16" t="n">
+      <c r="K16" t="n">
         <v>0.4457</v>
       </c>
-      <c r="K16" t="n">
-        <v>0.6431</v>
-      </c>
       <c r="L16" t="n">
-        <v>0.5265</v>
+        <v>0.5908</v>
       </c>
       <c r="M16" t="n">
-        <v>0.7504999999999999</v>
+        <v>0.5081</v>
       </c>
       <c r="N16" t="n">
-        <v>0.7259</v>
+        <v>0.7451</v>
       </c>
       <c r="O16" t="n">
-        <v>0.738</v>
+        <v>0.7075</v>
       </c>
       <c r="P16" t="n">
-        <v>0.8456</v>
+        <v>0.7258</v>
       </c>
     </row>
     <row r="17">
@@ -1338,31 +1349,31 @@
         <v>1614</v>
       </c>
       <c r="H17" t="n">
+        <v>3539</v>
+      </c>
+      <c r="I17" t="n">
         <v>3365</v>
       </c>
-      <c r="I17" t="n">
+      <c r="J17" t="n">
         <v>2737</v>
       </c>
-      <c r="J17" t="n">
+      <c r="K17" t="n">
         <v>0.5212</v>
       </c>
-      <c r="K17" t="n">
-        <v>0.6171</v>
-      </c>
       <c r="L17" t="n">
-        <v>0.5651</v>
+        <v>0.5449000000000001</v>
       </c>
       <c r="M17" t="n">
-        <v>0.7934</v>
+        <v>0.5328000000000001</v>
       </c>
       <c r="N17" t="n">
-        <v>0.6962</v>
+        <v>0.7805</v>
       </c>
       <c r="O17" t="n">
-        <v>0.7416</v>
+        <v>0.6732</v>
       </c>
       <c r="P17" t="n">
-        <v>0.8607</v>
+        <v>0.7229</v>
       </c>
     </row>
     <row r="18">
@@ -1392,31 +1403,31 @@
         <v>170</v>
       </c>
       <c r="H18" t="n">
+        <v>428</v>
+      </c>
+      <c r="I18" t="n">
         <v>537</v>
       </c>
-      <c r="I18" t="n">
+      <c r="J18" t="n">
         <v>535</v>
       </c>
-      <c r="J18" t="n">
+      <c r="K18" t="n">
         <v>0.6208</v>
       </c>
-      <c r="K18" t="n">
-        <v>0.6657999999999999</v>
-      </c>
       <c r="L18" t="n">
-        <v>0.6425</v>
+        <v>0.6213</v>
       </c>
       <c r="M18" t="n">
-        <v>0.8482</v>
+        <v>0.6211</v>
       </c>
       <c r="N18" t="n">
-        <v>0.7202</v>
+        <v>0.8374</v>
       </c>
       <c r="O18" t="n">
-        <v>0.779</v>
+        <v>0.7055</v>
       </c>
       <c r="P18" t="n">
-        <v>0.8572</v>
+        <v>0.7658</v>
       </c>
     </row>
     <row r="19">
@@ -1446,31 +1457,31 @@
         <v>390</v>
       </c>
       <c r="H19" t="n">
+        <v>1062</v>
+      </c>
+      <c r="I19" t="n">
         <v>2558</v>
       </c>
-      <c r="I19" t="n">
+      <c r="J19" t="n">
         <v>908</v>
       </c>
-      <c r="J19" t="n">
+      <c r="K19" t="n">
         <v>0.4274</v>
       </c>
-      <c r="K19" t="n">
-        <v>0.631</v>
-      </c>
       <c r="L19" t="n">
-        <v>0.5096000000000001</v>
+        <v>0.5783</v>
       </c>
       <c r="M19" t="n">
-        <v>0.739</v>
+        <v>0.4915</v>
       </c>
       <c r="N19" t="n">
-        <v>0.7095</v>
+        <v>0.7342</v>
       </c>
       <c r="O19" t="n">
-        <v>0.7239</v>
+        <v>0.6919999999999999</v>
       </c>
       <c r="P19" t="n">
-        <v>0.8295</v>
+        <v>0.7125</v>
       </c>
     </row>
     <row r="20">
@@ -1500,31 +1511,31 @@
         <v>485</v>
       </c>
       <c r="H20" t="n">
+        <v>1126</v>
+      </c>
+      <c r="I20" t="n">
         <v>1921</v>
       </c>
-      <c r="I20" t="n">
+      <c r="J20" t="n">
         <v>958</v>
       </c>
-      <c r="J20" t="n">
+      <c r="K20" t="n">
         <v>0.4593</v>
       </c>
-      <c r="K20" t="n">
-        <v>0.6181</v>
-      </c>
       <c r="L20" t="n">
-        <v>0.527</v>
+        <v>0.5538999999999999</v>
       </c>
       <c r="M20" t="n">
-        <v>0.7593</v>
+        <v>0.5022</v>
       </c>
       <c r="N20" t="n">
-        <v>0.6947</v>
+        <v>0.7513</v>
       </c>
       <c r="O20" t="n">
-        <v>0.7255</v>
+        <v>0.6744</v>
       </c>
       <c r="P20" t="n">
-        <v>0.8378</v>
+        <v>0.7108</v>
       </c>
     </row>
     <row r="21">
@@ -1554,31 +1565,31 @@
         <v>320</v>
       </c>
       <c r="H21" t="n">
+        <v>954</v>
+      </c>
+      <c r="I21" t="n">
         <v>1710</v>
       </c>
-      <c r="I21" t="n">
+      <c r="J21" t="n">
         <v>1144</v>
       </c>
-      <c r="J21" t="n">
+      <c r="K21" t="n">
         <v>0.4914</v>
       </c>
-      <c r="K21" t="n">
-        <v>0.5915</v>
-      </c>
       <c r="L21" t="n">
-        <v>0.5368000000000001</v>
+        <v>0.5508999999999999</v>
       </c>
       <c r="M21" t="n">
-        <v>0.7781</v>
+        <v>0.5195</v>
       </c>
       <c r="N21" t="n">
-        <v>0.6643</v>
+        <v>0.7713</v>
       </c>
       <c r="O21" t="n">
-        <v>0.7167</v>
+        <v>0.653</v>
       </c>
       <c r="P21" t="n">
-        <v>0.8178</v>
+        <v>0.7073</v>
       </c>
     </row>
   </sheetData>
@@ -1592,53 +1603,43 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>fold</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>fold_name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>test_case_series</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>strict_F1_mean</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>strict_F1_std</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>ade_F1_mean</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>ade_F1_std</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>detection_F1_mean</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>detection_F1_std</t>
         </is>
       </c>
     </row>
@@ -1657,22 +1658,16 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0.628</v>
+        <v>0.6002</v>
       </c>
       <c r="E2" t="n">
-        <v>0.009900000000000001</v>
+        <v>0.0114</v>
       </c>
       <c r="F2" t="n">
-        <v>0.7925</v>
+        <v>0.7733</v>
       </c>
       <c r="G2" t="n">
         <v>0.0092</v>
-      </c>
-      <c r="H2" t="n">
-        <v>0.8751</v>
-      </c>
-      <c r="I2" t="n">
-        <v>0.0108</v>
       </c>
     </row>
     <row r="3">
@@ -1690,22 +1685,16 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0.5602</v>
+        <v>0.5289</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0095</v>
+        <v>0.009299999999999999</v>
       </c>
       <c r="F3" t="n">
-        <v>0.7427</v>
+        <v>0.7242</v>
       </c>
       <c r="G3" t="n">
-        <v>0.0051</v>
-      </c>
-      <c r="H3" t="n">
-        <v>0.8643999999999999</v>
-      </c>
-      <c r="I3" t="n">
-        <v>0.0069</v>
+        <v>0.0036</v>
       </c>
     </row>
     <row r="4">
@@ -1723,22 +1712,16 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0.6563</v>
+        <v>0.6367</v>
       </c>
       <c r="E4" t="n">
-        <v>0.02</v>
+        <v>0.0201</v>
       </c>
       <c r="F4" t="n">
-        <v>0.7873</v>
+        <v>0.7751</v>
       </c>
       <c r="G4" t="n">
-        <v>0.013</v>
-      </c>
-      <c r="H4" t="n">
-        <v>0.8619</v>
-      </c>
-      <c r="I4" t="n">
-        <v>0.0073</v>
+        <v>0.0128</v>
       </c>
     </row>
     <row r="5">
@@ -1756,22 +1739,16 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>0.5274</v>
+        <v>0.5084</v>
       </c>
       <c r="E5" t="n">
-        <v>0.0112</v>
+        <v>0.0122</v>
       </c>
       <c r="F5" t="n">
-        <v>0.7239</v>
+        <v>0.7126</v>
       </c>
       <c r="G5" t="n">
-        <v>0.008999999999999999</v>
-      </c>
-      <c r="H5" t="n">
-        <v>0.829</v>
-      </c>
-      <c r="I5" t="n">
-        <v>0.0131</v>
+        <v>0.0077</v>
       </c>
     </row>
   </sheetData>
@@ -1789,27 +1766,27 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>category</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>strict_F1_mean</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>strict_F1_std</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>ade_F1_mean</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>ade_F1_std</t>
         </is>
@@ -2022,44 +1999,6 @@
       </c>
       <c r="E12" t="n">
         <v>0.0319</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>strict_f1_95ci</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>ade_f1_95ci</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>(0.5758, 0.5921)</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>(0.7543, 0.7649)</t>
-        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>